<commit_message>
feat: add Biology and Geology, THE EARTH and Vital Functions to the catalog
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -381,7 +381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="4" min="1" max="1"/>
@@ -731,6 +731,43 @@
         <is>
           <t>active</t>
         </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Biología y Geología</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Biología y Geología</v>
+      </c>
+      <c r="D7" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="E7"/>
+      <c r="F7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Actividades de repaso de biología y geología.</v>
+      </c>
+      <c r="H7" t="str">
+        <v>#6552A0</v>
+      </c>
+      <c r="I7" t="str">
+        <v>#EFEBF8</v>
+      </c>
+      <c r="J7" t="str">
+        <v>leaf</v>
+      </c>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7"/>
+      <c r="O7" t="str">
+        <v>active</v>
       </c>
     </row>
   </sheetData>
@@ -1777,7 +1814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:T34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="4" min="1" max="1"/>
@@ -3716,6 +3753,54 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>topic-biologia-geologia-the-earth</v>
+      </c>
+      <c r="B34" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="C34" t="str">
+        <v>THE EARTH</v>
+      </c>
+      <c r="D34" t="str">
+        <v>the-earth</v>
+      </c>
+      <c r="E34"/>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="str">
+        <v>La Tierra, los seres vivos y su organización.</v>
+      </c>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34" t="str">
+        <v>/images/topics/topic-biologia-geologia-the-earth.webp</v>
+      </c>
+      <c r="K34" t="str">
+        <v>La curvatura de la Tierra y sus luces nocturnas bajo un cielo estrellado.</v>
+      </c>
+      <c r="L34" t="str">
+        <v>50% 50%</v>
+      </c>
+      <c r="M34" t="str">
+        <v>credit-the-earth-tawatchai07</v>
+      </c>
+      <c r="N34" t="str">
+        <v>active</v>
+      </c>
+      <c r="O34"/>
+      <c r="P34"/>
+      <c r="Q34"/>
+      <c r="R34"/>
+      <c r="S34" t="str">
+        <v>globe-2</v>
+      </c>
+      <c r="T34" t="str">
+        <v>cover</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4011,7 +4096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="4" min="1" max="1"/>
@@ -4300,6 +4385,20 @@
       </c>
       <c r="D14" t="n">
         <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>actividad-interactiva</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Actividad interactiva</v>
+      </c>
+      <c r="C15" t="str">
+        <v>mouse-pointer-click</v>
+      </c>
+      <c r="D15" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -4411,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL83"/>
+  <dimension ref="A1:AL84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -16569,6 +16668,86 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>native-vital-functions</v>
+      </c>
+      <c r="B84" t="str">
+        <v>vital-functions</v>
+      </c>
+      <c r="C84"/>
+      <c r="D84" t="str">
+        <v>VITAL FUNCTIONS</v>
+      </c>
+      <c r="E84"/>
+      <c r="F84" t="str">
+        <v>Repasa las funciones vitales, la organización de los seres vivos y las biomoléculas con 11 ejercicios de selección, ordenación y clasificación.</v>
+      </c>
+      <c r="G84" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="H84" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="I84" t="str">
+        <v>topic-biologia-geologia-the-earth</v>
+      </c>
+      <c r="J84" t="str">
+        <v>en</v>
+      </c>
+      <c r="K84" t="str">
+        <v>actividad-interactiva</v>
+      </c>
+      <c r="L84" t="str">
+        <v>1.º ESO</v>
+      </c>
+      <c r="M84" t="str">
+        <v>funciones vitales | biomoléculas</v>
+      </c>
+      <c r="N84" t="str">
+        <v>vital functions | living things | organisms | organic | inorganic | nutrition | respiration | growth</v>
+      </c>
+      <c r="O84" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="P84" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="Q84" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="R84" t="str">
+        <v>published</v>
+      </c>
+      <c r="S84" t="str">
+        <v>native</v>
+      </c>
+      <c r="T84"/>
+      <c r="U84"/>
+      <c r="V84"/>
+      <c r="W84"/>
+      <c r="X84"/>
+      <c r="Y84"/>
+      <c r="Z84"/>
+      <c r="AA84"/>
+      <c r="AB84"/>
+      <c r="AC84"/>
+      <c r="AD84"/>
+      <c r="AE84"/>
+      <c r="AF84"/>
+      <c r="AG84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH84" t="str">
+        <v>mixed-practice</v>
+      </c>
+      <c r="AI84" t="str">
+        <v>data/native/vital-functions.json</v>
+      </c>
+      <c r="AJ84"/>
+      <c r="AK84"/>
+      <c r="AL84"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16580,7 +16759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="4" min="1" max="1"/>
@@ -18478,6 +18657,17 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>native-vital-functions</v>
+      </c>
+      <c r="B95" t="str">
+        <v>topic-biologia-geologia-the-earth</v>
+      </c>
+      <c r="C95"/>
+      <c r="D95"/>
+      <c r="E95"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -18489,7 +18679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="4" min="1" max="1"/>
@@ -19596,6 +19786,30 @@
         <is>
           <t xml:space="preserve">Generada/preparada el 2026-09-24. PNG original: topic-matematicas-operaciones-combinadas.png; SHA-256 1bc5bb2138465a33820974e4024a4329a1ee2a95de9eb1c969a6f04c82bd6da5. WebP 1600×900: ebf9e1625820896fd11cd5d191addb3399385fdd48bb595fecbd938366b06247. </t>
         </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>credit-the-earth-tawatchai07</v>
+      </c>
+      <c r="B34" t="str">
+        <v>THE EARTH — Tierra y galaxia</v>
+      </c>
+      <c r="C34" t="str">
+        <v>tawatchai07</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Imagen de tawatchai07 en Magnific</v>
+      </c>
+      <c r="E34" t="str">
+        <v>https://www.magnific.com/es/foto-gratis/tierra-galaxia-elementos-imagen-proporcionados-nasa_13180419.htm</v>
+      </c>
+      <c r="F34" t="str">
+        <v>No especificada en el material facilitado; consultar la fuente.</v>
+      </c>
+      <c r="G34"/>
+      <c r="H34" t="str">
+        <v>Imagen y atribución facilitadas por Alejandro Castaño Medina. EXIF: Earth and galaxy. Elements of this image furnished by NASA. Conversión local a WebP sin cambiar la composición.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(catalog): integrate Living Things Are Formed of Cells with regression coverage
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -4510,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL84"/>
+  <dimension ref="A1:AL85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -16748,6 +16748,86 @@
       <c r="AK84"/>
       <c r="AL84"/>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>native-living-things-are-formed-of-cells</v>
+      </c>
+      <c r="B85" t="str">
+        <v>living-things-are-formed-of-cells</v>
+      </c>
+      <c r="C85"/>
+      <c r="D85" t="str">
+        <v>LIVING THINGS ARE FORMED OF CELLS</v>
+      </c>
+      <c r="E85"/>
+      <c r="F85" t="str">
+        <v>Repasa las necesidades de los seres vivos, el descubrimiento de las células y los organismos unicelulares y multicelulares con ocho ejercicios interactivos.</v>
+      </c>
+      <c r="G85" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="H85" t="str">
+        <v>biologia-geologia</v>
+      </c>
+      <c r="I85" t="str">
+        <v>topic-biologia-geologia-the-earth</v>
+      </c>
+      <c r="J85" t="str">
+        <v>en</v>
+      </c>
+      <c r="K85" t="str">
+        <v>actividad-interactiva</v>
+      </c>
+      <c r="L85" t="str">
+        <v>1.º ESO</v>
+      </c>
+      <c r="M85" t="str">
+        <v>células | seres vivos</v>
+      </c>
+      <c r="N85" t="str">
+        <v>living things | cells | unicellular | multicellular | Leeuwenhoek | Hooke</v>
+      </c>
+      <c r="O85" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="P85" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="Q85" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="R85" t="str">
+        <v>published</v>
+      </c>
+      <c r="S85" t="str">
+        <v>native</v>
+      </c>
+      <c r="T85"/>
+      <c r="U85"/>
+      <c r="V85"/>
+      <c r="W85"/>
+      <c r="X85"/>
+      <c r="Y85"/>
+      <c r="Z85"/>
+      <c r="AA85"/>
+      <c r="AB85"/>
+      <c r="AC85"/>
+      <c r="AD85"/>
+      <c r="AE85"/>
+      <c r="AF85"/>
+      <c r="AG85" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH85" t="str">
+        <v>mixed-practice</v>
+      </c>
+      <c r="AI85" t="str">
+        <v>data/native/living-things-are-formed-of-cells.json</v>
+      </c>
+      <c r="AJ85"/>
+      <c r="AK85"/>
+      <c r="AL85"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16759,7 +16839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="4" min="1" max="1"/>
@@ -18667,6 +18747,17 @@
       <c r="C95"/>
       <c r="D95"/>
       <c r="E95"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>native-living-things-are-formed-of-cells</v>
+      </c>
+      <c r="B96" t="str">
+        <v>topic-biologia-geologia-the-earth</v>
+      </c>
+      <c r="C96"/>
+      <c r="D96"/>
+      <c r="E96"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add eight interactive activities to The Earth
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -88,6 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -734,40 +735,53 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Biología y Geología</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Biología y Geología</v>
-      </c>
-      <c r="D7" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="E7"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Biología y Geología</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Biología y Geología</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
       <c r="F7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" t="str">
-        <v>Actividades de repaso de biología y geología.</v>
-      </c>
-      <c r="H7" t="str">
-        <v>#6552A0</v>
-      </c>
-      <c r="I7" t="str">
-        <v>#EFEBF8</v>
-      </c>
-      <c r="J7" t="str">
-        <v>leaf</v>
-      </c>
-      <c r="K7"/>
-      <c r="L7"/>
-      <c r="M7"/>
-      <c r="N7"/>
-      <c r="O7" t="str">
-        <v>active</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Actividades de repaso de biología y geología.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>#6552A0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>#EFEBF8</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3754,51 +3768,68 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="str">
-        <v>topic-biologia-geologia-the-earth</v>
-      </c>
-      <c r="B34" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="C34" t="str">
-        <v>THE EARTH</v>
-      </c>
-      <c r="D34" t="str">
-        <v>the-earth</v>
-      </c>
-      <c r="E34"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>THE EARTH</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>the-earth</t>
+        </is>
+      </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
-      <c r="G34" t="str">
-        <v>La Tierra, los seres vivos y su organización.</v>
-      </c>
-      <c r="H34"/>
-      <c r="I34"/>
-      <c r="J34" t="str">
-        <v>/images/topics/topic-biologia-geologia-the-earth.webp</v>
-      </c>
-      <c r="K34" t="str">
-        <v>La curvatura de la Tierra y sus luces nocturnas bajo un cielo estrellado.</v>
-      </c>
-      <c r="L34" t="str">
-        <v>50% 50%</v>
-      </c>
-      <c r="M34" t="str">
-        <v>credit-the-earth-tawatchai07</v>
-      </c>
-      <c r="N34" t="str">
-        <v>active</v>
-      </c>
-      <c r="O34"/>
-      <c r="P34"/>
-      <c r="Q34"/>
-      <c r="R34"/>
-      <c r="S34" t="str">
-        <v>globe-2</v>
-      </c>
-      <c r="T34" t="str">
-        <v>cover</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>La Tierra, los seres vivos y su organización.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>/images/topics/topic-biologia-geologia-the-earth.webp</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>La curvatura de la Tierra y sus luces nocturnas bajo un cielo estrellado.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>50% 50%</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>credit-the-earth-tawatchai07</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>globe-2</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>cover</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4388,14 +4419,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
-        <v>actividad-interactiva</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Actividad interactiva</v>
-      </c>
-      <c r="C15" t="str">
-        <v>mouse-pointer-click</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Actividad interactiva</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>mouse-pointer-click</t>
+        </is>
       </c>
       <c r="D15" t="n">
         <v>14</v>
@@ -4412,7 +4449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -4499,6 +4536,31 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>lumi</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Lumi</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>app.lumi.education</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>#5b58c9</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4510,7 +4572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL85"/>
+  <dimension ref="A1:AM93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -4548,6 +4610,7 @@
     <col width="24" customWidth="1" style="4" min="33" max="33"/>
     <col width="30" customWidth="1" style="4" min="34" max="34"/>
     <col width="45" customWidth="1" style="4" min="35" max="35"/>
+    <col width="48" customWidth="1" style="4" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="4">
@@ -4741,6 +4804,11 @@
           <t>ID de crédito</t>
         </is>
       </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>URL de inserción</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -16669,164 +16737,1132 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="str">
-        <v>native-vital-functions</v>
-      </c>
-      <c r="B84" t="str">
-        <v>vital-functions</v>
-      </c>
-      <c r="C84"/>
-      <c r="D84" t="str">
-        <v>VITAL FUNCTIONS</v>
-      </c>
-      <c r="E84"/>
-      <c r="F84" t="str">
-        <v>Repasa las funciones vitales, la organización de los seres vivos y las biomoléculas con 11 ejercicios de selección, ordenación y clasificación.</v>
-      </c>
-      <c r="G84" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="H84" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="I84" t="str">
-        <v>topic-biologia-geologia-the-earth</v>
-      </c>
-      <c r="J84" t="str">
-        <v>en</v>
-      </c>
-      <c r="K84" t="str">
-        <v>actividad-interactiva</v>
-      </c>
-      <c r="L84" t="str">
-        <v>1.º ESO</v>
-      </c>
-      <c r="M84" t="str">
-        <v>funciones vitales | biomoléculas</v>
-      </c>
-      <c r="N84" t="str">
-        <v>vital functions | living things | organisms | organic | inorganic | nutrition | respiration | growth</v>
-      </c>
-      <c r="O84" t="str">
-        <v>2026-10-01</v>
-      </c>
-      <c r="P84" t="str">
-        <v>2026-10-01</v>
-      </c>
-      <c r="Q84" t="str">
-        <v>2026-10-01</v>
-      </c>
-      <c r="R84" t="str">
-        <v>published</v>
-      </c>
-      <c r="S84" t="str">
-        <v>native</v>
-      </c>
-      <c r="T84"/>
-      <c r="U84"/>
-      <c r="V84"/>
-      <c r="W84"/>
-      <c r="X84"/>
-      <c r="Y84"/>
-      <c r="Z84"/>
-      <c r="AA84"/>
-      <c r="AB84"/>
-      <c r="AC84"/>
-      <c r="AD84"/>
-      <c r="AE84"/>
-      <c r="AF84"/>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>native-vital-functions</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>vital-functions</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>VITAL FUNCTIONS</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Repasa las funciones vitales, la organización de los seres vivos y las biomoléculas con 11 ejercicios de selección, ordenación y clasificación.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>funciones vitales | biomoléculas</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>vital functions | living things | organisms | organic | inorganic | nutrition | respiration | growth</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
       <c r="AG84" t="n">
         <v>1</v>
       </c>
-      <c r="AH84" t="str">
-        <v>mixed-practice</v>
-      </c>
-      <c r="AI84" t="str">
-        <v>data/native/vital-functions.json</v>
-      </c>
-      <c r="AJ84"/>
-      <c r="AK84"/>
-      <c r="AL84"/>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>mixed-practice</t>
+        </is>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>data/native/vital-functions.json</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" t="str">
-        <v>native-living-things-are-formed-of-cells</v>
-      </c>
-      <c r="B85" t="str">
-        <v>living-things-are-formed-of-cells</v>
-      </c>
-      <c r="C85"/>
-      <c r="D85" t="str">
-        <v>LIVING THINGS ARE FORMED OF CELLS</v>
-      </c>
-      <c r="E85"/>
-      <c r="F85" t="str">
-        <v>Repasa las necesidades de los seres vivos, el descubrimiento de las células y los organismos unicelulares y multicelulares con ocho ejercicios interactivos.</v>
-      </c>
-      <c r="G85" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="H85" t="str">
-        <v>biologia-geologia</v>
-      </c>
-      <c r="I85" t="str">
-        <v>topic-biologia-geologia-the-earth</v>
-      </c>
-      <c r="J85" t="str">
-        <v>en</v>
-      </c>
-      <c r="K85" t="str">
-        <v>actividad-interactiva</v>
-      </c>
-      <c r="L85" t="str">
-        <v>1.º ESO</v>
-      </c>
-      <c r="M85" t="str">
-        <v>células | seres vivos</v>
-      </c>
-      <c r="N85" t="str">
-        <v>living things | cells | unicellular | multicellular | Leeuwenhoek | Hooke</v>
-      </c>
-      <c r="O85" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="P85" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="Q85" t="str">
-        <v>2026-10-03</v>
-      </c>
-      <c r="R85" t="str">
-        <v>published</v>
-      </c>
-      <c r="S85" t="str">
-        <v>native</v>
-      </c>
-      <c r="T85"/>
-      <c r="U85"/>
-      <c r="V85"/>
-      <c r="W85"/>
-      <c r="X85"/>
-      <c r="Y85"/>
-      <c r="Z85"/>
-      <c r="AA85"/>
-      <c r="AB85"/>
-      <c r="AC85"/>
-      <c r="AD85"/>
-      <c r="AE85"/>
-      <c r="AF85"/>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>native-living-things-are-formed-of-cells</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>living-things-are-formed-of-cells</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>LIVING THINGS ARE FORMED OF CELLS</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Repasa las necesidades de los seres vivos, el descubrimiento de las células y los organismos unicelulares y multicelulares con ocho ejercicios interactivos.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>células | seres vivos</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>living things | cells | unicellular | multicellular | Leeuwenhoek | Hooke</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
       <c r="AG85" t="n">
         <v>1</v>
       </c>
-      <c r="AH85" t="str">
-        <v>mixed-practice</v>
-      </c>
-      <c r="AI85" t="str">
-        <v>data/native/living-things-are-formed-of-cells.json</v>
-      </c>
-      <c r="AJ85"/>
-      <c r="AK85"/>
-      <c r="AL85"/>
+      <c r="AH85" t="inlineStr">
+        <is>
+          <t>mixed-practice</t>
+        </is>
+      </c>
+      <c r="AI85" t="inlineStr">
+        <is>
+          <t>data/native/living-things-are-formed-of-cells.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>EP-30815160</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>what-are-cells-like-animal-and-plant-cell</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>What Are Cells Like? Animal and Plant Cell</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>What Are Cells Like? Animal and Plant Cell</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P86" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q86" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>educaplay</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>30815160</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30815160-what_are_cells_like.html</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30815160-what_are_cells_like.html</t>
+        </is>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30815160-what_are_cells_like.html</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA86" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB86" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM86" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/juego/30815160-what_are_cells_like.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>EP-30945103</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>animal-cell</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Animal Cell</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Animal Cell</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P87" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q87" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>educaplay</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>30945103</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30945103-animal_cell.html</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30945103-animal_cell.html</t>
+        </is>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/30945103-animal_cell.html</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA87" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM87" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/juego/30945103-animal_cell.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>EP-31000797</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>plant-cell</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Plant Cell</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Plant Cell</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P88" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q88" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>educaplay</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>31000797</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/31000797-eukaryotic_cel.html</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/31000797-eukaryotic_cel.html</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/recursos-educativos/31000797-eukaryotic_cel.html</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA88" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB88" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM88" t="inlineStr">
+        <is>
+          <t>https://es.educaplay.com/juego/31000797-eukaryotic_cel.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>LUMI-1PCQ0H</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>how-do-living-things-get-nutrients</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>How Do Living Things Get Nutrients?</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>How Do Living Things Get Nutrients?</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P89" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q89" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>lumi</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>1PCQ0H</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/1PCQ0H</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/1PCQ0H</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/1PCQ0H</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA89" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB89" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM89" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/1PCQ0H</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>LUMI-IUQRTE</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>how-do-living-things-reproduce-part-1</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>How Do Living Things Reproduce? Parte 1</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>How Do Living Things Reproduce? Parte 1</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P90" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q90" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>lumi</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>iuQrtE</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/iuQrtE</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/iuQrtE</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/iuQrtE</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA90" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB90" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/iuQrtE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>WW-121629558</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>how-do-living-things-reproduce-part-2</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>How Do Living Things Reproduce? Parte 2</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>How Do Living Things Reproduce? Parte 2</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P91" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q91" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>wordwall</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>121629558</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121629558?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121629558?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121629558?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA91" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB91" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM91" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/embed/fc0b8b174f2b466f80b7f879d3e72e14?themeId=1&amp;templateId=2&amp;fontStackId=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>LUMI-3ARRY5</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>how-do-living-things-interact-with-their-environment-part-1</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>How Do Living Things Interact with Their Environment? Parte 1</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>How Do Living Things Interact with Their Environment? Parte 1</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P92" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q92" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>lumi</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>3Arry5</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/3Arry5</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/3Arry5</t>
+        </is>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/3Arry5</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA92" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB92" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM92" t="inlineStr">
+        <is>
+          <t>https://app.lumi.education/run/3Arry5</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>WW-121676126</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>how-do-living-things-interact-with-their-environment-part-2</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>How Do Living Things Interact with Their Environment? Parte 2</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>How Do Living Things Interact with Their Environment? Parte 2</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>biologia-geologia</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>actividad-interactiva</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Curso de origen desconocido</t>
+        </is>
+      </c>
+      <c r="P93" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="Q93" s="7" t="n">
+        <v>46313</v>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>external</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>wordwall</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>121676126</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121676126?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121676126?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/resource/121676126?wwmethod=link</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="AA93" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB93" t="inlineStr">
+        <is>
+          <t>Markdown proporcionado</t>
+        </is>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
+        </is>
+      </c>
+      <c r="AM93" t="inlineStr">
+        <is>
+          <t>https://wordwall.net/embed/66f02bba25bd48fdbabe4bd91dec5d23?themeId=1&amp;templateId=2&amp;fontStackId=0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16839,7 +17875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="4" min="1" max="1"/>
@@ -18738,26 +19774,124 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="str">
-        <v>native-vital-functions</v>
-      </c>
-      <c r="B95" t="str">
-        <v>topic-biologia-geologia-the-earth</v>
-      </c>
-      <c r="C95"/>
-      <c r="D95"/>
-      <c r="E95"/>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>native-vital-functions</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" t="str">
-        <v>native-living-things-are-formed-of-cells</v>
-      </c>
-      <c r="B96" t="str">
-        <v>topic-biologia-geologia-the-earth</v>
-      </c>
-      <c r="C96"/>
-      <c r="D96"/>
-      <c r="E96"/>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>native-living-things-are-formed-of-cells</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>EP-30815160</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>EP-30945103</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>EP-31000797</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>LUMI-1PCQ0H</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>LUMI-IUQRTE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>WW-121629558</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>LUMI-3ARRY5</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>WW-121676126</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>topic-biologia-geologia-the-earth</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19880,27 +21014,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="str">
-        <v>credit-the-earth-tawatchai07</v>
-      </c>
-      <c r="B34" t="str">
-        <v>THE EARTH — Tierra y galaxia</v>
-      </c>
-      <c r="C34" t="str">
-        <v>tawatchai07</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Imagen de tawatchai07 en Magnific</v>
-      </c>
-      <c r="E34" t="str">
-        <v>https://www.magnific.com/es/foto-gratis/tierra-galaxia-elementos-imagen-proporcionados-nasa_13180419.htm</v>
-      </c>
-      <c r="F34" t="str">
-        <v>No especificada en el material facilitado; consultar la fuente.</v>
-      </c>
-      <c r="G34"/>
-      <c r="H34" t="str">
-        <v>Imagen y atribución facilitadas por Alejandro Castaño Medina. EXIF: Earth and galaxy. Elements of this image furnished by NASA. Conversión local a WebP sin cambiar la composición.</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>credit-the-earth-tawatchai07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>THE EARTH — Tierra y galaxia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>tawatchai07</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Imagen de tawatchai07 en Magnific</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.magnific.com/es/foto-gratis/tierra-galaxia-elementos-imagen-proporcionados-nasa_13180419.htm</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>No especificada en el material facilitado; consultar la fuente.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Imagen y atribución facilitadas por Alejandro Castaño Medina. EXIF: Earth and galaxy. Elements of this image furnished by NASA. Conversión local a WebP sin cambiar la composición.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: set The Earth course to 1 ESO
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -16984,7 +16984,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P86" s="7" t="n">
@@ -17100,7 +17100,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P87" s="7" t="n">
@@ -17216,7 +17216,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P88" s="7" t="n">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P89" s="7" t="n">
@@ -17448,7 +17448,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P90" s="7" t="n">
@@ -17564,7 +17564,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P91" s="7" t="n">
@@ -17680,7 +17680,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P92" s="7" t="n">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>Curso de origen desconocido</t>
+          <t>1.º ESO</t>
         </is>
       </c>
       <c r="P93" s="7" t="n">

</xml_diff>

<commit_message>
data: describe The Earth interactive activities
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -16957,6 +16957,11 @@
           <t>What Are Cells Like? Animal and Plant Cell</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>English-language quiz with questions about cells and the characteristics of animal and plant cells.</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -16985,6 +16990,16 @@
       <c r="L86" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>animal cell | plant cell | cell structure</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>célula animal | célula vegetal | eukaryotic cell | cells | cell parts</t>
         </is>
       </c>
       <c r="P86" s="7" t="n">
@@ -17073,6 +17088,11 @@
           <t>Animal Cell</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>English-language interactive map for identifying the parts of an animal cell and reviewing eukaryotic cell structure.</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17101,6 +17121,16 @@
       <c r="L87" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>animal cell | eukaryotic cell | cell parts</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>célula animal | célula eucariota | cell structure | organelles | interactive map</t>
         </is>
       </c>
       <c r="P87" s="7" t="n">
@@ -17189,6 +17219,11 @@
           <t>Plant Cell</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>English-language interactive map to identify the parts of a plant cell and review eukaryotic cell structure.</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17217,6 +17252,16 @@
       <c r="L88" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>plant cell | eukaryotic cell | cell parts</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>célula vegetal | célula eucariota | cell structure | organelles | interactive map</t>
         </is>
       </c>
       <c r="P88" s="7" t="n">
@@ -17305,6 +17350,11 @@
           <t>How Do Living Things Get Nutrients?</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>English-language quiz on the nutrition function in living things, including autotrophic and heterotrophic nutrition, nutrients, cellular respiration and the route oxygen follows through the body.</t>
+        </is>
+      </c>
       <c r="G89" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17333,6 +17383,16 @@
       <c r="L89" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>cellular nutrition | autotrophic nutrition | heterotrophic nutrition</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>nutrición celular | nutrients | cell respiration | mitochondria | oxygen pathway | nutrición autótrofa | nutrición heterótrofa</t>
         </is>
       </c>
       <c r="P89" s="7" t="n">
@@ -17421,6 +17481,11 @@
           <t>How Do Living Things Reproduce? Parte 1</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>English-language quiz on mitosis and cell reproduction, comparing asexual and sexual reproduction and reviewing chromosome numbers in female cells and embryos.</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17449,6 +17514,16 @@
       <c r="L90" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>mitosis | asexual reproduction | sexual reproduction</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>mitosis | reproducción asexual | reproducción sexual | chromosomes | chromosomes in cells | embryo</t>
         </is>
       </c>
       <c r="P90" s="7" t="n">
@@ -17537,6 +17612,11 @@
           <t>How Do Living Things Reproduce? Parte 2</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>English-language group-sort activity to classify features and examples of sexual and asexual reproduction, including sex cells, zygotes, plants, animals and unicellular organisms.</t>
+        </is>
+      </c>
       <c r="G91" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17565,6 +17645,16 @@
       <c r="L91" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>sexual reproduction | asexual reproduction | reproduction examples</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>reproducción sexual | reproducción asexual | gametes | sex cells | zygote | unicellular organisms | classification</t>
         </is>
       </c>
       <c r="P91" s="7" t="n">
@@ -17653,6 +17743,11 @@
           <t>How Do Living Things Interact with Their Environment? Parte 1</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>English-language quiz on the interaction function: how cells respond to stimuli and move by amoeboid, contractile or vibratile mechanisms involving pseudopodia, cilia and flagella.</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17681,6 +17776,16 @@
       <c r="L92" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>interaction function | cell movement | response to stimuli</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>función de relación | movimiento celular | amoeboid movement | pseudopodia | cilia | flagella | contractile movement</t>
         </is>
       </c>
       <c r="P92" s="7" t="n">
@@ -17769,6 +17874,11 @@
           <t>How Do Living Things Interact with Their Environment? Parte 2</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>English-language group-sort activity to classify cellular movement mechanisms and their features: amoeboid, contractile, ciliary and flagellar movement.</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr">
         <is>
           <t>biologia-geologia</t>
@@ -17797,6 +17907,16 @@
       <c r="L93" t="inlineStr">
         <is>
           <t>1.º ESO</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>interaction function | cell movement | types of movement</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>función de relación | movimiento celular | pseudopodia | cilia | flagella | contractile movement | classification</t>
         </is>
       </c>
       <c r="P93" s="7" t="n">

</xml_diff>